<commit_message>
Added Claim Points testcases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7F2C868-B2B2-434A-AD06-D1BD8F3CB3D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C2C0DDC-D7FE-46B8-B2BE-003A64EA6E7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="18">
   <si>
     <t>MODULE</t>
   </si>
@@ -45,28 +45,40 @@
     <t>FEATURE</t>
   </si>
   <si>
-    <t>Login</t>
-  </si>
-  <si>
     <t>CompanyLogin</t>
   </si>
   <si>
-    <t>CompanyLoginTest.xlsx</t>
-  </si>
-  <si>
     <t>NO</t>
   </si>
   <si>
-    <t>DirectLogin.xlsx</t>
-  </si>
-  <si>
     <t>ClaimPoints</t>
   </si>
   <si>
     <t>YES</t>
   </si>
   <si>
-    <t>MyClaimsPageTest.xlsx</t>
+    <t>01_Login</t>
+  </si>
+  <si>
+    <t>02_ClaimPoints</t>
+  </si>
+  <si>
+    <t>01_DirectLogin.xlsx</t>
+  </si>
+  <si>
+    <t>01_CompanyLoginTest.xlsx</t>
+  </si>
+  <si>
+    <t>02_InfluencerLogin.xlsx</t>
+  </si>
+  <si>
+    <t>01_MyClaimsPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>02_DealerPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>03_CategoryPageTest.xlsx</t>
   </si>
 </sst>
 </file>
@@ -398,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="23.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="23.6328125" customWidth="1"/>
@@ -423,16 +435,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>4</v>
@@ -440,16 +452,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>4</v>
@@ -457,18 +469,69 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Created Category Page & Cart Details testcases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C2C0DDC-D7FE-46B8-B2BE-003A64EA6E7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43EFE85-2C7F-4783-85F4-101FA0052F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="20">
   <si>
     <t>MODULE</t>
   </si>
@@ -79,6 +79,12 @@
   </si>
   <si>
     <t>03_CategoryPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>04_ClaimInformationPageTest</t>
+  </si>
+  <si>
+    <t>05_AddClaimTest</t>
   </si>
 </sst>
 </file>
@@ -110,12 +116,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -124,10 +145,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -410,10 +431,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultColWidth="23.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="23.6328125" customWidth="1"/>
+    <col min="4" max="4" width="29.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -520,7 +541,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>11</v>
@@ -532,6 +553,40 @@
         <v>17</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Test Cases files of Claim Modules
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43EFE85-2C7F-4783-85F4-101FA0052F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB230D50-0C07-4590-B398-7AA0407BB641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="19">
   <si>
     <t>MODULE</t>
   </si>
@@ -54,9 +54,6 @@
     <t>ClaimPoints</t>
   </si>
   <si>
-    <t>YES</t>
-  </si>
-  <si>
     <t>01_Login</t>
   </si>
   <si>
@@ -81,10 +78,10 @@
     <t>03_CategoryPageTest.xlsx</t>
   </si>
   <si>
-    <t>04_ClaimInformationPageTest</t>
-  </si>
-  <si>
-    <t>05_AddClaimTest</t>
+    <t>04_ClaimInformationPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>05_AddClaimTest.xlsx</t>
   </si>
 </sst>
 </file>
@@ -459,13 +456,13 @@
         <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>4</v>
@@ -476,13 +473,13 @@
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>4</v>
@@ -493,13 +490,13 @@
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>4</v>
@@ -510,13 +507,13 @@
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>4</v>
@@ -527,13 +524,13 @@
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>4</v>
@@ -544,13 +541,13 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>4</v>
@@ -558,16 +555,16 @@
     </row>
     <row r="8" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>4</v>
@@ -578,13 +575,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Added Test Cases Excution flow of REdemption module
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -5,27 +5,38 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12483A8C-B220-445A-A175-53B78EAAF41F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF798D7-9FB9-439D-BE9D-C589E1D33F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="380" windowWidth="19200" windowHeight="9190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Execution" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="30">
   <si>
     <t>MODULE</t>
   </si>
@@ -94,6 +105,27 @@
   </si>
   <si>
     <t>05_AddClaimTest.xlsx</t>
+  </si>
+  <si>
+    <t>04_Redemptions</t>
+  </si>
+  <si>
+    <t>Redemptions</t>
+  </si>
+  <si>
+    <t>01_RedemptionHistoryPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>02_RewardCataloguePageTest.xlsx</t>
+  </si>
+  <si>
+    <t>03_RedemptionCartPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>04_RedemptionSummaryPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>05_AddRedemptionTest.xlsx</t>
   </si>
 </sst>
 </file>
@@ -450,10 +482,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="23.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="23.6328125" customWidth="1"/>
+    <col min="4" max="4" width="36.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -474,7 +506,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -491,7 +523,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -525,7 +557,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -542,7 +574,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -559,7 +591,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -575,8 +607,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -593,7 +625,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -610,8 +642,8 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>9</v>
+      <c r="A10" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>18</v>
@@ -623,6 +655,91 @@
         <v>20</v>
       </c>
       <c r="E10" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Call Me & Reward Catalogue Module TestCases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF798D7-9FB9-439D-BE9D-C589E1D33F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1161FCD6-948D-479F-92D9-F21D32051293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="42">
   <si>
     <t>MODULE</t>
   </si>
@@ -126,6 +126,42 @@
   </si>
   <si>
     <t>05_AddRedemptionTest.xlsx</t>
+  </si>
+  <si>
+    <t>05_CallMe</t>
+  </si>
+  <si>
+    <t>CallMe</t>
+  </si>
+  <si>
+    <t>01_CallMeTest.xlsx</t>
+  </si>
+  <si>
+    <t>DigitalBusinessCard</t>
+  </si>
+  <si>
+    <t>01_DigitalBusinessCardTest.xlsx</t>
+  </si>
+  <si>
+    <t>06_RewardCatalogue</t>
+  </si>
+  <si>
+    <t>RewardCatalogue</t>
+  </si>
+  <si>
+    <t>01_RewardCataloguePageTest.xlsx</t>
+  </si>
+  <si>
+    <t>02_RedemptionCartPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>03_RedemptionSummaryPageTest.xlsx</t>
+  </si>
+  <si>
+    <t>04_AddRedemptionTest.xlsx</t>
+  </si>
+  <si>
+    <t>07_DigitalBusinessCard</t>
   </si>
 </sst>
 </file>
@@ -164,7 +200,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -187,11 +223,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -200,6 +260,15 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="23.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="36.26953125" customWidth="1"/>
@@ -676,7 +745,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -693,7 +762,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -710,8 +779,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>9</v>
+      <c r="A14" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>23</v>
@@ -727,7 +796,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -740,6 +809,108 @@
         <v>29</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added  Digital Business card Scenarios
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1161FCD6-948D-479F-92D9-F21D32051293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0466BD25-0FB7-4454-905A-BF05BE4C5218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="48">
   <si>
     <t>MODULE</t>
   </si>
@@ -162,6 +162,24 @@
   </si>
   <si>
     <t>07_DigitalBusinessCard</t>
+  </si>
+  <si>
+    <t>08_SendBusinessCard</t>
+  </si>
+  <si>
+    <t>SendBusinessCard</t>
+  </si>
+  <si>
+    <t>01_SendBusinessCardTest.xlsx</t>
+  </si>
+  <si>
+    <t>09_MyWebSite</t>
+  </si>
+  <si>
+    <t>MyWebSite</t>
+  </si>
+  <si>
+    <t>01_MyWebSiteTest.xlsx</t>
   </si>
 </sst>
 </file>
@@ -251,7 +269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -269,6 +287,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -551,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="23.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="36.26953125" customWidth="1"/>
@@ -899,7 +923,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>41</v>
@@ -911,6 +935,37 @@
         <v>34</v>
       </c>
       <c r="E21" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B23" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" s="8" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Master Excution File Updated
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -31,7 +31,7 @@
     <t>SHEET</t>
   </si>
   <si>
-    <t>NO</t>
+    <t>YES</t>
   </si>
   <si>
     <t>01_Login</t>
@@ -77,6 +77,9 @@
     <t>05_AddClaimTest.xlsx</t>
   </si>
   <si>
+    <t>NO</t>
+  </si>
+  <si>
     <t>03_Profile</t>
   </si>
   <si>
@@ -141,9 +144,6 @@
   </si>
   <si>
     <t>01_DigitalBusinessCardTest.xlsx</t>
-  </si>
-  <si>
-    <t>YES</t>
   </si>
   <si>
     <t>08_SendBusinessCard</t>
@@ -686,7 +686,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A7" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>13</v>
@@ -737,16 +737,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A10" s="3" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>9</v>
@@ -757,13 +757,13 @@
         <v>5</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>9</v>
@@ -774,13 +774,13 @@
         <v>5</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>9</v>
@@ -791,13 +791,13 @@
         <v>5</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>9</v>
@@ -808,13 +808,13 @@
         <v>5</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>9</v>
@@ -825,30 +825,30 @@
         <v>5</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="20.25" customFormat="1" s="1">
       <c r="A16" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>9</v>
@@ -859,13 +859,13 @@
         <v>5</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>9</v>
@@ -876,13 +876,13 @@
         <v>5</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>9</v>
@@ -893,13 +893,13 @@
         <v>5</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>9</v>
@@ -910,13 +910,13 @@
         <v>5</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>9</v>
@@ -927,13 +927,13 @@
         <v>5</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>9</v>
@@ -941,7 +941,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A22" s="5" t="s">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>43</v>
@@ -958,7 +958,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A23" s="5" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>46</v>

</xml_diff>

<commit_message>
testng.xml  and MasterExecution file update
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A741FB84-8D3F-430E-A44D-3860344D040D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Execution" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Execution"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -37,24 +31,27 @@
     <t>SHEET</t>
   </si>
   <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>01_Login</t>
+  </si>
+  <si>
+    <t>CompanyLogin</t>
+  </si>
+  <si>
+    <t>01_CompanyLoginTest.xlsx</t>
+  </si>
+  <si>
+    <t>TestCases</t>
+  </si>
+  <si>
+    <t>02_InfluencerLogin.xlsx</t>
+  </si>
+  <si>
     <t>NO</t>
   </si>
   <si>
-    <t>01_Login</t>
-  </si>
-  <si>
-    <t>CompanyLogin</t>
-  </si>
-  <si>
-    <t>01_CompanyLoginTest.xlsx</t>
-  </si>
-  <si>
-    <t>TestCases</t>
-  </si>
-  <si>
-    <t>02_InfluencerLogin.xlsx</t>
-  </si>
-  <si>
     <t>01_DirectLogin.xlsx</t>
   </si>
   <si>
@@ -170,9 +167,6 @@
   </si>
   <si>
     <t>01_MyHealthBenefitsTest.xlsx</t>
-  </si>
-  <si>
-    <t>YES</t>
   </si>
   <si>
     <t>11_KYCSubmission</t>
@@ -229,8 +223,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -251,6 +246,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -260,7 +261,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -307,63 +308,42 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="8">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -374,10 +354,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -415,71 +395,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -507,7 +487,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -530,11 +510,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -543,13 +523,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -559,7 +539,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -568,7 +548,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -577,7 +557,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -585,10 +565,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -653,21 +633,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22" style="6" customWidth="1"/>
+    <col min="1" max="1" style="7" width="8.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="17.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="33.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="22.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -684,7 +664,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -701,7 +681,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -718,9 +698,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A4" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -729,468 +709,468 @@
         <v>7</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="C7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="C8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A13" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="C13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="C14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A15" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="C15" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A16" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A17" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A18" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="C18" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A19" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>32</v>
-      </c>
       <c r="C19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A20" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>32</v>
-      </c>
       <c r="C20" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A21" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="7" t="s">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A22" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="C22" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E22" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" s="7" t="s">
+      <c r="D22" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="E22" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A23" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="C23" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" s="7" t="s">
+      <c r="D23" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="E23" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A24" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="C24" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" s="7" t="s">
+      <c r="D24" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A25" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E25" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" s="7" t="s">
+      <c r="E25" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A26" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B27" s="7" t="s">
+      <c r="E26" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A27" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E27" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B28" s="7" t="s">
+      <c r="E27" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A28" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E28" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B29" s="8" t="s">
+      <c r="E28" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A29" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B30" s="8" t="s">
+      <c r="E29" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25" customFormat="1" s="1">
+      <c r="A30" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B31" s="8" t="s">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25" customFormat="1" s="1">
+      <c r="A31" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="6" t="s">
         <v>67</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Master Execution File IUpdate
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -225,7 +225,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,12 +243,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -312,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -329,11 +323,8 @@
     <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -640,11 +631,11 @@
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="8.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="17.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="33.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="8.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="17.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="33.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="22.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="33" customFormat="1" s="1">
@@ -1106,7 +1097,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A28" s="3" t="s">
         <v>5</v>
       </c>
@@ -1123,54 +1114,54 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="33" customFormat="1" s="1">
-      <c r="A29" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B29" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A29" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25" customFormat="1" s="1">
-      <c r="A30" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B30" s="6" t="s">
+      <c r="A30" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="3" t="s">
         <v>66</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25" customFormat="1" s="1">
-      <c r="A31" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B31" s="6" t="s">
+      <c r="A31" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="3" t="s">
         <v>67</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update My Website Module Resubmit TestCases - 11-Jun-2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="69">
   <si>
     <t>EXECUTE</t>
   </si>
@@ -157,7 +157,10 @@
     <t>MyWebSite</t>
   </si>
   <si>
-    <t>01_MyWebSiteTest.xlsx</t>
+    <t>01_WebSite_Add.xlsx</t>
+  </si>
+  <si>
+    <t>02_WebSite_Resubmit.xlsx</t>
   </si>
   <si>
     <t>10_MyHealthBenefits</t>
@@ -628,7 +631,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="6" width="8.290714285714287" customWidth="1" bestFit="1"/>
@@ -655,7 +658,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -672,7 +675,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -689,7 +692,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -706,7 +709,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
@@ -723,7 +726,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
@@ -740,7 +743,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -757,7 +760,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
@@ -774,7 +777,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A9" s="3" t="s">
         <v>5</v>
       </c>
@@ -910,7 +913,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A17" s="4" t="s">
         <v>5</v>
       </c>
@@ -927,7 +930,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A18" s="4" t="s">
         <v>5</v>
       </c>
@@ -944,7 +947,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A19" s="4" t="s">
         <v>5</v>
       </c>
@@ -961,7 +964,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A20" s="4" t="s">
         <v>5</v>
       </c>
@@ -995,7 +998,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="33" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A22" s="3" t="s">
         <v>5</v>
       </c>
@@ -1034,13 +1037,13 @@
         <v>5</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>9</v>
@@ -1051,13 +1054,13 @@
         <v>5</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>9</v>
@@ -1068,13 +1071,13 @@
         <v>5</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>56</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>9</v>
@@ -1085,13 +1088,13 @@
         <v>5</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>9</v>
@@ -1102,13 +1105,13 @@
         <v>5</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>9</v>
@@ -1119,33 +1122,33 @@
         <v>5</v>
       </c>
       <c r="B29" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="E29" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A30" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="C30" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25" customFormat="1" s="1">
-      <c r="A30" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>64</v>
-      </c>
       <c r="D30" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>66</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25" customFormat="1" s="1">
@@ -1153,16 +1156,33 @@
         <v>5</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>67</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25" customFormat="1" s="1">
+      <c r="A32" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CostCalculator Module TestCases Updated
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACA7E61-2F5F-4A33-968C-23C149E0CD2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Execution"/>
+    <sheet name="Execution" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="67">
   <si>
     <t>EXECUTE</t>
   </si>
@@ -215,19 +221,12 @@
   </si>
   <si>
     <t>01_CostCalculatorTest.xlsx</t>
-  </si>
-  <si>
-    <t>TestCalculationsCase1</t>
-  </si>
-  <si>
-    <t>TestCalculationsCase2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -258,7 +257,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -305,39 +304,92 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -348,10 +400,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -389,71 +441,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -481,7 +533,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -504,11 +556,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -517,13 +569,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -533,7 +585,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -542,7 +594,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -551,7 +603,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -559,10 +611,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -627,21 +679,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="6" width="8.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="17.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="33.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="8.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="33" customFormat="1" s="1">
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -658,9 +710,9 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="2" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -675,9 +727,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="3" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
@@ -692,7 +744,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="4" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -709,9 +761,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="5" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>13</v>
@@ -726,9 +778,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="6" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>13</v>
@@ -743,9 +795,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="7" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>13</v>
@@ -760,9 +812,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="8" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>13</v>
@@ -777,9 +829,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="9" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>13</v>
@@ -794,9 +846,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="33" customFormat="1" s="1">
+    <row r="10" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>20</v>
@@ -811,9 +863,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="33" customFormat="1" s="1">
+    <row r="11" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>23</v>
@@ -828,9 +880,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="12" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>23</v>
@@ -845,9 +897,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="13" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>23</v>
@@ -862,9 +914,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="14" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>23</v>
@@ -879,9 +931,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="15" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>23</v>
@@ -896,9 +948,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="16" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>30</v>
@@ -913,9 +965,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="17" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>33</v>
@@ -930,9 +982,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="18" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>33</v>
@@ -947,9 +999,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="33" customFormat="1" s="1">
+    <row r="19" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>33</v>
@@ -964,9 +1016,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="20" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>33</v>
@@ -981,9 +1033,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="33" customFormat="1" s="1">
+    <row r="21" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>39</v>
@@ -998,9 +1050,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="22" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>42</v>
@@ -1015,9 +1067,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="23" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>45</v>
@@ -1032,9 +1084,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="24" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>45</v>
@@ -1049,9 +1101,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="25" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>49</v>
@@ -1066,9 +1118,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="26" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>52</v>
@@ -1083,9 +1135,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="27" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>55</v>
@@ -1100,9 +1152,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="28" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>58</v>
@@ -1117,9 +1169,9 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5" customFormat="1" s="1">
-      <c r="A29" s="3" t="s">
-        <v>5</v>
+    <row r="29" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>61</v>
@@ -1134,55 +1186,21 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5" customFormat="1" s="1">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="9" t="s">
         <v>64</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E30" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25" customFormat="1" s="1">
-      <c r="A31" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25" customFormat="1" s="1">
-      <c r="A32" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>68</v>
+      <c r="E30" s="8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update CostCalculator Module testcases - 16-Jun-2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACA7E61-2F5F-4A33-968C-23C149E0CD2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4371BD52-B042-42A8-9AA4-741DEE4B1E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -711,8 +711,8 @@
       </c>
     </row>
     <row r="2" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>11</v>
+      <c r="A2" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -728,8 +728,8 @@
       </c>
     </row>
     <row r="3" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>11</v>
+      <c r="A3" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
@@ -762,8 +762,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>11</v>
+      <c r="A5" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>13</v>
@@ -779,8 +779,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>11</v>
+      <c r="A6" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>13</v>
@@ -796,8 +796,8 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>11</v>
+      <c r="A7" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>13</v>
@@ -813,8 +813,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>11</v>
+      <c r="A8" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>13</v>
@@ -830,8 +830,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>11</v>
+      <c r="A9" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>13</v>
@@ -847,8 +847,8 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>11</v>
+      <c r="A10" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>20</v>
@@ -864,8 +864,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>11</v>
+      <c r="A11" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>23</v>
@@ -881,8 +881,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>11</v>
+      <c r="A12" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>23</v>
@@ -898,8 +898,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>11</v>
+      <c r="A13" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>23</v>
@@ -915,8 +915,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>11</v>
+      <c r="A14" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>23</v>
@@ -932,8 +932,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>11</v>
+      <c r="A15" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>23</v>
@@ -949,8 +949,8 @@
       </c>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>11</v>
+      <c r="A16" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>30</v>
@@ -966,8 +966,8 @@
       </c>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
-        <v>11</v>
+      <c r="A17" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>33</v>
@@ -983,8 +983,8 @@
       </c>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
-        <v>11</v>
+      <c r="A18" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>33</v>
@@ -1000,8 +1000,8 @@
       </c>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
-        <v>11</v>
+      <c r="A19" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>33</v>
@@ -1017,8 +1017,8 @@
       </c>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
-        <v>11</v>
+      <c r="A20" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>33</v>
@@ -1034,8 +1034,8 @@
       </c>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>11</v>
+      <c r="A21" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>39</v>
@@ -1051,8 +1051,8 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
-        <v>11</v>
+      <c r="A22" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>42</v>
@@ -1068,8 +1068,8 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
-        <v>11</v>
+      <c r="A23" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>45</v>
@@ -1085,8 +1085,8 @@
       </c>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
-        <v>11</v>
+      <c r="A24" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>45</v>
@@ -1102,8 +1102,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
-        <v>11</v>
+      <c r="A25" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>49</v>
@@ -1119,8 +1119,8 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
-        <v>11</v>
+      <c r="A26" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>52</v>
@@ -1136,7 +1136,7 @@
       </c>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B27" s="3" t="s">
@@ -1153,8 +1153,8 @@
       </c>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="3" t="s">
-        <v>11</v>
+      <c r="A28" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>58</v>
@@ -1170,8 +1170,8 @@
       </c>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="4" t="s">
-        <v>11</v>
+      <c r="A29" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Resolved Failed Test cases - 19-Jun-2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/MasterExecution.xlsx
+++ b/src/test/resources/testdata/MasterExecution.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4371BD52-B042-42A8-9AA4-741DEE4B1E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Execution" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Execution"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -226,8 +220,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -239,6 +234,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -257,7 +258,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -305,17 +306,15 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -324,19 +323,6 @@
         <color rgb="FF000000"/>
       </left>
       <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -350,46 +336,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -400,10 +383,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -441,71 +424,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -533,7 +516,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -556,11 +539,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -569,13 +552,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -585,7 +568,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -594,7 +577,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -603,7 +586,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -611,10 +594,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -679,21 +662,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E30"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="9" width="8.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="9" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="9" width="17.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="9" width="33.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="9" width="22.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -710,496 +693,496 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="E2" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="E3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
+      <c r="E4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
+      <c r="E5" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="s">
+      <c r="E6" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3" t="s">
+      <c r="E7" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="3" t="s">
+      <c r="E8" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="3" t="s">
+      <c r="E9" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A10" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="E10" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="3" t="s">
+      <c r="E11" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="3" t="s">
+      <c r="E12" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A13" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="3" t="s">
+      <c r="E13" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="3" t="s">
+      <c r="E14" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A15" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" s="3" t="s">
+      <c r="E15" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A16" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" s="4" t="s">
+      <c r="E16" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A17" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" s="3" t="s">
+      <c r="E17" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A18" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="3" t="s">
+      <c r="E18" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="3" t="s">
+      <c r="E19" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="4" t="s">
+      <c r="E20" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="33" customFormat="1" s="1">
+      <c r="A21" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" s="3" t="s">
+      <c r="E21" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A22" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E22" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" s="3" t="s">
+      <c r="E22" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A23" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" s="3" t="s">
+      <c r="E23" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A24" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" s="3" t="s">
+      <c r="E24" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A25" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" s="3" t="s">
+      <c r="E25" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A26" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" s="3" t="s">
+      <c r="E26" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A27" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B28" s="3" t="s">
+      <c r="E27" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A28" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E28" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B29" s="3" t="s">
+      <c r="E28" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="A29" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B30" s="9" t="s">
+      <c r="E29" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A30" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="3" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>